<commit_message>
con electrica y sistemas
</commit_message>
<xml_diff>
--- a/clasificacion_saberes/output/personas_saberes_comision.xlsx
+++ b/clasificacion_saberes/output/personas_saberes_comision.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repositories\profes\clasificacion_saberes\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CAD12B4D-EC8E-4086-BC88-D8A0E19CA817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E3B6D9-84BA-4A26-AB31-1607C9EBF590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{3BEC65EA-4C49-41AB-9DD1-333D80F94044}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{3BEC65EA-4C49-41AB-9DD1-333D80F94044}"/>
   </bookViews>
   <sheets>
     <sheet name="personas_saberes_comision" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="154">
   <si>
     <t>codigo</t>
   </si>
@@ -37,18 +37,12 @@
     <t>Alberto Garro Zavaleta</t>
   </si>
   <si>
-    <t>DTE;GAE;GCV;GEE;IEM</t>
-  </si>
-  <si>
     <t>COZ0</t>
   </si>
   <si>
     <t>Carlos Otárola Zúñiga</t>
   </si>
   <si>
-    <t>CIM;EDM;MAN;MSF;TTC</t>
-  </si>
-  <si>
     <t>CVS0</t>
   </si>
   <si>
@@ -67,18 +61,12 @@
     <t>Frank Marín Guillén</t>
   </si>
   <si>
-    <t>IYT</t>
-  </si>
-  <si>
     <t>GMJ0</t>
   </si>
   <si>
     <t>Gonzalo Mora Jiménez</t>
   </si>
   <si>
-    <t>CEE;IYT;MEE;GEE</t>
-  </si>
-  <si>
     <t>GBG0</t>
   </si>
   <si>
@@ -118,9 +106,6 @@
     <t>Ignacio del Valle Granados</t>
   </si>
   <si>
-    <t>LID;MSF</t>
-  </si>
-  <si>
     <t>JMJ0</t>
   </si>
   <si>
@@ -139,18 +124,12 @@
     <t>Juan Pablo Arias Cartín</t>
   </si>
   <si>
-    <t>MAN;DTE;GAE;GCV;GEE;IEM</t>
-  </si>
-  <si>
     <t>JRG0</t>
   </si>
   <si>
     <t>Julio César Rojas Gómez</t>
   </si>
   <si>
-    <t>MSF</t>
-  </si>
-  <si>
     <t>LSM0</t>
   </si>
   <si>
@@ -163,18 +142,12 @@
     <t>Lisandro Araya Rodriguez</t>
   </si>
   <si>
-    <t>CEE;IYT;MEE</t>
-  </si>
-  <si>
     <t>LMC0</t>
   </si>
   <si>
     <t>Luis Carlos Muñoz Chacón</t>
   </si>
   <si>
-    <t>LID;CEE;IYT;MEE</t>
-  </si>
-  <si>
     <t>LMS0</t>
   </si>
   <si>
@@ -199,9 +172,6 @@
     <t>Manuel Francisco Mata Coto</t>
   </si>
   <si>
-    <t>IPR;CIM;EDM;MAN;MSF;TTC;DTE;GAE;GCV;GEE;IEM</t>
-  </si>
-  <si>
     <t>NVP0</t>
   </si>
   <si>
@@ -220,21 +190,12 @@
     <t>Oscar Monge Ruiz</t>
   </si>
   <si>
-    <t>LID;DTE;GAE;GCV;GEE;IEM</t>
-  </si>
-  <si>
     <t>OGC0</t>
   </si>
   <si>
     <t>Osvaldo Guerrero Castro</t>
   </si>
   <si>
-    <t>REH0</t>
-  </si>
-  <si>
-    <t>Rodolfo Elizondo Hernandez</t>
-  </si>
-  <si>
     <t>RMC0</t>
   </si>
   <si>
@@ -247,24 +208,12 @@
     <t>Sebastián Mata Ortega</t>
   </si>
   <si>
-    <t>SMC0</t>
-  </si>
-  <si>
-    <t>Suzanne Melara Cruz</t>
-  </si>
-  <si>
-    <t>LID;CEE;DTE;GAE;GCV;GEE;IEM</t>
-  </si>
-  <si>
     <t>VJH0</t>
   </si>
   <si>
     <t>Víctor Julio Hernández</t>
   </si>
   <si>
-    <t>ACP;AME;MSF</t>
-  </si>
-  <si>
     <t>DPI;IYT;CIM;MSF;EDM;MYS;MNC</t>
   </si>
   <si>
@@ -316,7 +265,223 @@
     <t>IEM;GEE</t>
   </si>
   <si>
-    <t>AQUI</t>
+    <t>Luis Chévez Gómez</t>
+  </si>
+  <si>
+    <t>LCG0</t>
+  </si>
+  <si>
+    <t>Marvin Bermúdez Chacón</t>
+  </si>
+  <si>
+    <t>MBC0</t>
+  </si>
+  <si>
+    <t>Maximino Jiménez Ceciliano</t>
+  </si>
+  <si>
+    <t>MJC0</t>
+  </si>
+  <si>
+    <t>DPI;MSF;MAN;EYD;MET</t>
+  </si>
+  <si>
+    <t>DPI;IEM</t>
+  </si>
+  <si>
+    <t>DPI</t>
+  </si>
+  <si>
+    <t>DPI;MSF;EDM;MAN</t>
+  </si>
+  <si>
+    <t>DPI;IYT;CIM;MSF;MAN;MNC</t>
+  </si>
+  <si>
+    <t>CEE;MEE;GAE;DTE</t>
+  </si>
+  <si>
+    <t>IEM</t>
+  </si>
+  <si>
+    <t>MSF;EDM;IEM</t>
+  </si>
+  <si>
+    <t>TTC;IEM;GEE</t>
+  </si>
+  <si>
+    <t>JMH0</t>
+  </si>
+  <si>
+    <t>Julio Andrés Morera Hidalgo</t>
+  </si>
+  <si>
+    <t>MSF;GEE</t>
+  </si>
+  <si>
+    <t>ADP;DPI;MSF;IEM</t>
+  </si>
+  <si>
+    <t>CEE;SCA</t>
+  </si>
+  <si>
+    <t>ADP;IEM;GAE;DTE</t>
+  </si>
+  <si>
+    <t>DPI;MSF;MAN</t>
+  </si>
+  <si>
+    <t>MSF;EDM</t>
+  </si>
+  <si>
+    <t>CEE;MAC;ASE</t>
+  </si>
+  <si>
+    <t>DPI;CIM;MSF;EDM;MNC</t>
+  </si>
+  <si>
+    <t>MEE;IEM;GEE</t>
+  </si>
+  <si>
+    <t>ADP;IEM;GEE</t>
+  </si>
+  <si>
+    <t>DPI;MSF;AME;GCA;SAA</t>
+  </si>
+  <si>
+    <t>CPS0</t>
+  </si>
+  <si>
+    <t>Carlos Piedra Santamaría</t>
+  </si>
+  <si>
+    <t>ADP;MAN;CDM;MET;IEM;GCV;GEE</t>
+  </si>
+  <si>
+    <t>DPI;MEE;IEM;GAE;DTE</t>
+  </si>
+  <si>
+    <t>SCA;IEM;GCV;GEE</t>
+  </si>
+  <si>
+    <t>MSF;TTC;IEM;GEE;ACP;GCA</t>
+  </si>
+  <si>
+    <t>ADP;CDM;IEM;GCV;GEE</t>
+  </si>
+  <si>
+    <t>ECV0</t>
+  </si>
+  <si>
+    <t>Erick Chinchilla Vargas</t>
+  </si>
+  <si>
+    <t>SFM0</t>
+  </si>
+  <si>
+    <t>Sofía Jimenez Monge</t>
+  </si>
+  <si>
+    <t>BMC0</t>
+  </si>
+  <si>
+    <t>Bryan Mesen Campos</t>
+  </si>
+  <si>
+    <t>DMH0</t>
+  </si>
+  <si>
+    <t>Diana Morales Hidalgo</t>
+  </si>
+  <si>
+    <t>NRQ0</t>
+  </si>
+  <si>
+    <t>Natalia Rojas Quesada</t>
+  </si>
+  <si>
+    <t>MSQ0</t>
+  </si>
+  <si>
+    <t>Marilyn Solano Quesada</t>
+  </si>
+  <si>
+    <t>ADP;CEE;IYT;MYS;SCA;ISC</t>
+  </si>
+  <si>
+    <t>HIP;IEM</t>
+  </si>
+  <si>
+    <t>AAV0</t>
+  </si>
+  <si>
+    <t>Alejandro Arroyo Valle</t>
+  </si>
+  <si>
+    <t>Ana Laura Loría</t>
+  </si>
+  <si>
+    <t>ALL0</t>
+  </si>
+  <si>
+    <t>AAG0</t>
+  </si>
+  <si>
+    <t>Andrés Arguello Guillén</t>
+  </si>
+  <si>
+    <t>AVH0</t>
+  </si>
+  <si>
+    <t>Anyelo Vargas Hernández</t>
+  </si>
+  <si>
+    <t>Carlos Montoya Marín</t>
+  </si>
+  <si>
+    <t>CMM0</t>
+  </si>
+  <si>
+    <t>Diego Gómez Rivera</t>
+  </si>
+  <si>
+    <t>DGR0</t>
+  </si>
+  <si>
+    <t>Emmanuel Muñoz Peña</t>
+  </si>
+  <si>
+    <t>EMP0</t>
+  </si>
+  <si>
+    <t>JBC0</t>
+  </si>
+  <si>
+    <t>Jenifer Brenes Casasola</t>
+  </si>
+  <si>
+    <t>Jose Miguel Ocampo Solano</t>
+  </si>
+  <si>
+    <t>JOS0</t>
+  </si>
+  <si>
+    <t>Luis Diego Araya Campos</t>
+  </si>
+  <si>
+    <t>LAC0</t>
+  </si>
+  <si>
+    <t>MJA0</t>
+  </si>
+  <si>
+    <t>María Jesús Amador Orozco</t>
+  </si>
+  <si>
+    <t>Sofia Madrigal Gamboa</t>
+  </si>
+  <si>
+    <t>MMG0</t>
   </si>
 </sst>
 </file>
@@ -861,9 +1026,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -901,7 +1066,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1007,7 +1172,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1149,7 +1314,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1157,7 +1322,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F4F652C-2260-48C5-8E69-8EE2DEC0370B}">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="49.36328125" customWidth="1"/>
@@ -1177,90 +1342,90 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -1271,155 +1436,205 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="C13" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>35</v>
+      </c>
+      <c r="C14" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>8</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>5</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" t="s">
         <v>37</v>
       </c>
-      <c r="B25" t="s">
-        <v>38</v>
-      </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" t="s">
         <v>45</v>
       </c>
-      <c r="B28" t="s">
-        <v>46</v>
-      </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -1430,51 +1645,51 @@
         <v>49</v>
       </c>
       <c r="C29" t="s">
-        <v>50</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>8</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B31" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>56</v>
+      </c>
+      <c r="B32" t="s">
         <v>57</v>
       </c>
-      <c r="B32" t="s">
-        <v>58</v>
-      </c>
       <c r="C32" t="s">
-        <v>59</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C33" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -1485,84 +1700,224 @@
         <v>63</v>
       </c>
       <c r="C34" t="s">
-        <v>8</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="C35" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="C37" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="C38" t="s">
-        <v>5</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B39" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="C39" t="s">
-        <v>5</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>75</v>
+        <v>116</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
+        <v>128</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>120</v>
+      </c>
+      <c r="B42" t="s">
+        <v>121</v>
+      </c>
+      <c r="C42" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>122</v>
+      </c>
+      <c r="B43" t="s">
+        <v>123</v>
+      </c>
+      <c r="C43" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>124</v>
+      </c>
+      <c r="B44" t="s">
+        <v>125</v>
+      </c>
+      <c r="C44" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>126</v>
+      </c>
+      <c r="B45" t="s">
+        <v>127</v>
+      </c>
+      <c r="C45" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>133</v>
+      </c>
+      <c r="B47" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>134</v>
+      </c>
+      <c r="B48" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>136</v>
+      </c>
+      <c r="B49" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>139</v>
+      </c>
+      <c r="B50" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>141</v>
+      </c>
+      <c r="B51" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>143</v>
+      </c>
+      <c r="B52" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>144</v>
+      </c>
+      <c r="B53" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>147</v>
+      </c>
+      <c r="B54" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>149</v>
+      </c>
+      <c r="B55" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>150</v>
+      </c>
+      <c r="B56" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>153</v>
+      </c>
+      <c r="B57" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>